<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-08 La feuille brune de Victorino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-08.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-08.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La feuille collée au lait</t>
+          <t>La feuille brune de Victorino</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin à la rosée, puis classe</t>
+          <t>cuisine au toast, classe, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, papa, maman, maîtresse</t>
+          <t>Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut montrer la feuille brune au petit trou. Le mot est déjà là. Il lève la main, il attend, puis il parle.</t>
+          <t>Le beurre fond. Le pain grillé saute. Sur le toast, un éclat de mie brille. Victorino veut montrer la feuille brune, maintenant. Il parle trop vite : les mots se perdent. Il saisit le toast : l'éclat saute. À la classe, il lève la feuille : personne ne regarde. Il refuse de foncer, lève la main, attend, puis dit. Merci vécu. L'éclat de mie tient sur le toast.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le banc du jardin a de la rosée. La bouteille de lait est froide. Une goutte glisse sur le verre. Une feuille brune est collée dessus. Elle s'est accrochée, Victorino. Elle fait crac. Victorino la décolle tout doucement. La feuille a un petit trou. On dirait une fenêtre. Une toute petite. Tu la mets dans la poche ? Oui. Pour l'école. Une petite bouchée, d'abord. Le pain est encore tiède. Le beurre fond un peu. C'est croustillant. On essuie tes doigts. Voilà. Le sac attend près du banc. Ta veste bleue. Les boutons, un par un. On marche. Dehors, d'autres feuilles font crac. Crac. Crac. Oui. On marche dessus. L'école a une porte rouge. Une petite cloche sonne une fois. La veste bleue reste au crochet. Au revoir, Victorino. Au revoir, maman. On revient. Tu ranges tes chaussures ? Oui, papa. En ce moment, Victorino s'assoit. Le tapis gris est un peu rêche. La feuille brune reste dans sa poche. Il la sent, tout contre le tissu. Bonjour. Bonjour. Qu'avez-vous trouvé dehors ? Victorino a une idée. Sa feuille brune. Le petit trou, comme une fenêtre. Le mot est déjà là. Il touche la poche. La maîtresse tient encore une pomme de pin. Elle la pose tout doucement.</t>
+          <t>Le beurre fond tout seul. La cuisine sent le toast chaud. Une assiette blanche attend sur la table. Le pain grillé saute dans l'assiette. Il saute, papa ! Tu l'entends, le petit bruit ? Sur le toast, un éclat de mie brille. Il brille, maman. C'est la mie, sous la lumière. Une feuille brune reste dans sa poche. Elle est sèche. Elle a un petit trou. Tu la montres à l'école ? Oui, papa. Maintenant ! En ce moment, Victorino saisit le toast. L'éclat de mie saute près de l'assiette. Ma feuille, papa ! Papa n'a pas fini sa phrase. Une petite bouchée, Victorino. Les deux voix se mélangent. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Tes doigts sont près de l'assiette ? Oui, papa. Papa se baisse à sa hauteur. On essuie tes doigts. Voilà. C'est croustillant. Un doigt reste un peu brillant. C'est le beurre, Victorino. Il est chaud. Le sac attend près du banc. Ta veste bleue. Les boutons, un par un. Les feuilles du jardin sont sèches. Ta veste est boutonnée ? Oui, papa. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, les feuilles font crac. Crac. Crac. On marche dessus. On marche sur le tapis de feuilles. L'école a une porte rouge. Une petite cloche sonne une fois. La veste bleue reste au crochet. Le couloir sent le savon. Une petite flaque brille sous la chaussure. On revient. Au revoir, papa. La veste est un peu chaude. Le tapis de la classe est gris. Victorino s'assoit, les genoux au tapis. Il sent le toast sur ses doigts. La feuille brune reste dans sa poche. Bonjour. Bonjour, maîtresse. Victorino a une idée. Sa feuille est brune, avec un trou. Je veux parler de la feuille ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne tourne la tête. Victorino referme la bouche. Il repose les mains sur ses genoux.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le banc du jardin a de la rosée. La bouteille de lait est froide. Une goutte glisse sur le verre. Une feuille brune est collée dessus. Elle s'est accrochée, Victorino. Elle fait crac. Victorino la décolle tout doucement. La feuille a un petit trou. On dirait une fenêtre. Une toute petite. Tu la mets dans la poche ? Oui. Pour l'école. Une petite bouchée, d'abord. Le pain est encore tiède. Le beurre fond un peu. C'est croustillant. On essuie tes doigts. Voilà. Le sac attend près du banc. Ta veste bleue. Les boutons, un par un. On marche. Dehors, d'autres feuilles font crac. Crac. Crac. Oui. On marche dessus. L'école a une porte rouge. Une petite cloche sonne une fois. La veste bleue reste au crochet. Au revoir, Victorino. Au revoir, maman. On revient. Tu ranges tes chaussures ? Oui, papa. En ce moment, Victorino s'assoit. Le tapis gris est un peu rêche. La feuille brune reste dans sa poche. Il la sent, tout contre le tissu. Bonjour. Bonjour. Qu'avez-vous trouvé dehors ? Victorino a une idée. Sa feuille brune. Le petit trou, comme une fenêtre. Le mot est déjà là. Il touche la poche. La maîtresse tient encore une pomme de pin. Elle la pose tout doucement.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le beurre fond tout seul. La cuisine sent le toast chaud. Une assiette blanche attend sur la table. Le pain grillé saute dans l'assiette. Il saute, papa ! Tu l'entends, le petit bruit ? Sur le toast, un &lt;emphasis level="moderate"&gt;éclat de mie&lt;/emphasis&gt; brille. Il brille, maman. C'est la mie, sous la lumière. Une feuille brune reste dans sa poche. Elle est sèche. Elle a un petit trou. Tu la montres à l'école ? Oui, papa. Maintenant ! En ce moment, Victorino saisit le toast. L'éclat de mie saute près de l'assiette. Ma feuille, papa ! Papa n'a pas fini sa phrase. Une petite bouchée, Victorino. Les deux voix se mélangent. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Tes doigts sont près de l'assiette ? Oui, papa. Papa se baisse à sa hauteur. On essuie tes doigts. Voilà. C'est croustillant. Un doigt reste un peu brillant. C'est le beurre, Victorino. Il est chaud. Le sac attend près du banc. Ta veste bleue. Les boutons, un par un. Les feuilles du jardin sont sèches. Ta veste est boutonnée ? Oui, papa. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, les feuilles font crac. Crac. Crac. On marche dessus. On marche sur le tapis de feuilles. L'école a une porte rouge. Une petite cloche sonne une fois. La veste bleue reste au crochet. Le couloir sent le savon. Une petite flaque brille sous la chaussure. On revient. Au revoir, papa. La veste est un peu chaude. Le tapis de la classe est gris. Victorino s'assoit, les genoux au tapis. Il sent le toast sur ses doigts. La feuille brune reste dans sa poche. Bonjour. Bonjour, maîtresse. Victorino a une idée. Sa feuille est brune, avec un trou. Je veux parler de la feuille ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne tourne la tête. Victorino referme la bouche. Il repose les mains sur ses genoux.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dorian arrive en classe. Maman dit au revoir. Dorian s'assoit. La maîtresse pose une question. Dorian a une idée. Il lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Dorian attend encore. Puis la maîtresse dit : Dorian. C'est ton tour. Dorian parle. Il dit : le chat est gris. Le soir, maman demande. Dorian dit : j'ai attendu. Puis j'ai parlé. Maman dit : merci. Attendre, puis parler.&lt;/slow&gt; [pause]</t>
+          <t>Le beurre fond tout seul. La cuisine sent le toast chaud. Une assiette blanche attend sur la table. Le pain grillé saute dans l'assiette. Il saute, papa ! Tu l'entends, le petit bruit ? Sur le toast, un &lt;emphasis&gt;éclat de mie&lt;/emphasis&gt; brille. Il brille, maman. C'est la mie, sous la lumière. Une feuille brune reste dans sa poche. Elle est sèche. Elle a un petit trou. Tu la montres à l'école ? Oui, papa. Maintenant ! En ce moment, Victorino saisit le toast. L'éclat de mie saute près de l'assiette. Ma feuille, papa ! Papa n'a pas fini sa phrase. Une petite bouchée, Victorino. Les deux voix se mélangent. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Tes doigts sont près de l'assiette ? Oui, papa. Papa se baisse à sa hauteur. On essuie tes doigts. Voilà. C'est croustillant. Un doigt reste un peu brillant. C'est le beurre, Victorino. Il est chaud. Le sac attend près du banc. Ta veste bleue. Les boutons, un par un. Les feuilles du jardin sont sèches. Ta veste est boutonnée ? Oui, papa. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, les feuilles font crac. Crac. Crac. On marche dessus. On marche sur le tapis de feuilles. L'école a une porte rouge. Une petite cloche sonne une fois. La veste bleue reste au crochet. Le couloir sent le savon. Une petite flaque brille sous la chaussure. On revient. Au revoir, papa. La veste est un peu chaude. Le tapis de la classe est gris. Victorino s'assoit, les genoux au tapis. Il sent le toast sur ses doigts. La feuille brune reste dans sa poche. Bonjour. Bonjour, maîtresse. Victorino a une idée. Sa feuille est brune, avec un trou. Je veux parler de la feuille ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne tourne la tête. Victorino referme la bouche. Il repose les mains sur ses genoux. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de mie</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,61 +1324,87 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_montrer_la_feuille_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le banc du jardin a de la rosée.
-narrateur|La bouteille de lait est froide.
-narrateur|Une goutte glisse sur le verre.
-narrateur|Une feuille brune est collée dessus.
-papa|Elle s'est accrochée, Victorino.
-enfant-m|Elle fait crac.
-narrateur|Victorino la décolle tout doucement.
-narrateur|La feuille a un petit trou.
-maman|On dirait une fenêtre.
-enfant-m|Une toute petite.
-papa|Tu la mets dans la poche ?
-enfant-m|Oui.
-enfant-m|Pour l'école.
-maman|Une petite bouchée, d'abord.
-narrateur|Le pain est encore tiède.
-narrateur|Le beurre fond un peu.
-enfant-m|C'est croustillant.
+          <t>narrateur|Le beurre fond tout seul.
+narrateur|La cuisine sent le toast chaud.
+narrateur|Une assiette blanche attend sur la table.
+narrateur|Le pain grillé saute dans l'assiette.
+enfant-m|Il saute, papa !
+papa|Tu l'entends, le petit bruit ?
+narrateur|Sur le toast, un éclat de mie brille.
+enfant-m|Il brille, maman.
+maman|C'est la mie, sous la lumière.
+narrateur|Une feuille brune reste dans sa poche.
+enfant-m|Elle est sèche.
+enfant-m|Elle a un petit trou.
+papa|Tu la montres à l'école ?
+enfant-m|Oui, papa.
+enfant-m|Maintenant !
+narrateur|En ce moment, Victorino saisit le toast.
+narrateur|L'éclat de mie saute près de l'assiette.
+enfant-m|Ma feuille, papa !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Une petite bouchée, Victorino.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Ça ne veut pas !
+papa|Tes doigts sont près de l'assiette ?
+enfant-m|Oui, papa.
+narrateur|Papa se baisse à sa hauteur.
 maman|On essuie tes doigts.
 maman|Voilà.
+enfant-m|C'est croustillant.
+narrateur|Un doigt reste un peu brillant.
+papa|C'est le beurre, Victorino.
+enfant-m|Il est chaud.
 narrateur|Le sac attend près du banc.
 maman|Ta veste bleue.
 maman|Les boutons, un par un.
-papa|On marche.
-narrateur|Dehors, d'autres feuilles font crac.
+papa|Les feuilles du jardin sont sèches.
+papa|Ta veste est boutonnée ?
+enfant-m|Oui, papa.
+papa|On y va ?
+enfant-m|On y va.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Victorino.
+narrateur|Dehors, les feuilles font crac.
 enfant-m|Crac.
 enfant-m|Crac.
-papa|Oui.
 papa|On marche dessus.
+narrateur|On marche sur le tapis de feuilles.
 narrateur|L'école a une porte rouge.
 narrateur|Une petite cloche sonne une fois.
 narrateur|La veste bleue reste au crochet.
-maman|Au revoir, Victorino.
-enfant-m|Au revoir, maman.
+narrateur|Le couloir sent le savon.
+narrateur|Une petite flaque brille sous la chaussure.
 papa|On revient.
-papa|Tu ranges tes chaussures ?
-enfant-m|Oui, papa.
-narrateur|En ce moment, Victorino s'assoit.
-narrateur|Le tapis gris est un peu rêche.
+enfant-m|Au revoir, papa.
+narrateur|La veste est un peu chaude.
+narrateur|Le tapis de la classe est gris.
+narrateur|Victorino s'assoit, les genoux au tapis.
+narrateur|Il sent le toast sur ses doigts.
 narrateur|La feuille brune reste dans sa poche.
-narrateur|Il la sent, tout contre le tissu.
 maitresse|Bonjour.
-enfant-m|Bonjour.
-maitresse|Qu'avez-vous trouvé dehors ?
+enfant-m|Bonjour, maîtresse.
 narrateur|Victorino a une idée.
-narrateur|Sa feuille brune.
-narrateur|Le petit trou, comme une fenêtre.
-narrateur|Le mot est déjà là.
-narrateur|Il touche la poche.
-narrateur|La maîtresse tient encore une pomme de pin.
-narrateur|Elle la pose tout doucement.</t>
+narrateur|Sa feuille est brune, avec un trou.
+enfant-m|Je veux parler de la feuille !
+narrateur|Il ouvre la bouche trop vite.
+narrateur|Ses mots se cognent à la classe.
+narrateur|Personne ne tourne la tête.
+narrateur|Victorino referme la bouche.
+narrateur|Il repose les mains sur ses genoux.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1415,12 +1441,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dorian veut parler. Que fait-il d'abord ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1483,7 +1509,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1491,10 +1517,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,34 +1535,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,13 +1575,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1561,7 +1591,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_leve_la_main_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1594,17 +1624,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino lève la main. Sa main reste en l'air. Il attend. Il sent la feuille dans sa poche. Sa main ne descend pas. Victorino. C'est toi. Tu peux parler. Ma feuille est brune. Elle fait crac. Elle a un petit trou. Il sort la feuille. Il la tient à deux mains. Une petite fenêtre, oui. Elle était sur le lait. Victorino lève la feuille. Un peu de lumière passe dans le trou. Merci, Victorino. Un cube jaune attend près du tapis. Victorino le regarde, sans le prendre. Le cube est lisse. La feuille reste dans sa main.</t>
+          <t>Victorino veut montrer la feuille, tout de suite. Ma feuille est brune ! Il lève la feuille trop vite. La feuille penche, puis retombe. Oh. Personne ne regarde la feuille. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Une main monte, sans crier. Sa main reste en l'air. Une autre voix parle d'un caillou. Victorino reste près de sa place. Il sent la feuille dans sa poche. Sur son doigt, l'éclat de mie brille. Sa main ne descend pas. Victorino. Un silence arrive, tout petit. Ma feuille est brune. Elle fait crac. Elle a un petit trou. Il sort la feuille, à deux mains. Un peu de lumière passe dans le trou. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Un cube jaune attend près du tapis. Victorino le regarde, sans le prendre. Le cube est lisse, un peu froid. Une petite fenêtre, oui. Le ventre de Victorino se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino lève la main. Sa main reste en l'air. Il attend. Il sent la feuille dans sa poche. Sa main ne descend pas. Victorino. C'est toi. Tu peux parler. Ma feuille est brune. Elle fait crac. Elle a un petit trou. Il sort la feuille. Il la tient à deux mains. Une petite fenêtre, oui. Elle était sur le lait. Victorino lève la feuille. Un peu de lumière passe dans le trou. Merci, Victorino. Un cube jaune attend près du tapis. Victorino le regarde, sans le prendre. Le cube est lisse. La feuille reste dans sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut montrer la feuille, tout de suite. Ma feuille est brune ! Il lève la feuille trop vite. La feuille penche, puis retombe. Oh. Personne ne regarde la feuille. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Une &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt; monte, sans crier. Sa main reste en l'air. Une autre voix parle d'un caillou. Victorino reste près de sa place. Il sent la feuille dans sa poche. Sur son doigt, l'éclat de mie brille. Sa main ne descend pas. Victorino. Un silence arrive, tout petit. Ma feuille est brune. Elle fait crac. Elle a un petit trou. Il sort la feuille, à deux mains. Un peu de lumière passe dans le trou. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Un cube jaune attend près du tapis. Victorino le regarde, sans le prendre. Le cube est lisse, un peu froid. Une petite fenêtre, oui. Le ventre de Victorino se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dorian a levé la main. Il a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; il a parlé. C'était son tour.&lt;/slow&gt; [pause]</t>
+          <t>Victorino veut montrer la feuille, tout de suite. Ma feuille est brune ! Il lève la feuille trop vite. La feuille penche, puis retombe. Oh. Personne ne regarde la feuille. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Une &lt;emphasis&gt;main&lt;/emphasis&gt; monte, sans crier. Sa main reste en l'air. Une autre voix parle d'un caillou. Victorino reste près de sa place. Il sent la feuille dans sa poche. Sur son doigt, l'éclat de mie brille. Sa main ne descend pas. Victorino. Un silence arrive, tout petit. Ma feuille est brune. Elle fait crac. Elle a un petit trou. Il sort la feuille, à deux mains. Un peu de lumière passe dans le trou. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Un cube jaune attend près du tapis. Victorino le regarde, sans le prendre. Le cube est lisse, un peu froid. Une petite fenêtre, oui. Le ventre de Victorino se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,18 +1681,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1685,30 +1715,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>main</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1747,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1729,37 +1759,50 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_dit_la_feuille_brune; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino lève la main.
+          <t>narrateur|Victorino veut montrer la feuille, tout de suite.
+enfant-m|Ma feuille est brune !
+narrateur|Il lève la feuille trop vite.
+narrateur|La feuille penche, puis retombe.
+enfant-m|Oh.
+narrateur|Personne ne regarde la feuille.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Une main monte, sans crier.
 narrateur|Sa main reste en l'air.
-narrateur|Il attend.
+narrateur|Une autre voix parle d'un caillou.
+narrateur|Victorino reste près de sa place.
 narrateur|Il sent la feuille dans sa poche.
+narrateur|Sur son doigt, l'éclat de mie brille.
 narrateur|Sa main ne descend pas.
 maitresse|Victorino.
-maitresse|C'est toi.
-maitresse|Tu peux parler.
+narrateur|Un silence arrive, tout petit.
 enfant-m|Ma feuille est brune.
 enfant-m|Elle fait crac.
 enfant-m|Elle a un petit trou.
-narrateur|Il sort la feuille.
-narrateur|Il la tient à deux mains.
-maitresse|Une petite fenêtre, oui.
-enfant-m|Elle était sur le lait.
-narrateur|Victorino lève la feuille.
+narrateur|Il sort la feuille, à deux mains.
 narrateur|Un peu de lumière passe dans le trou.
-maitresse|Merci, Victorino.
+narrateur|Une tête se tourne vers lui.
+narrateur|Les oreilles écoutent jusqu'au bout.
 narrateur|Un cube jaune attend près du tapis.
 narrateur|Victorino le regarde, sans le prendre.
-narrateur|Le cube est lisse.
-narrateur|La feuille reste dans sa main.</t>
+narrateur|Le cube est lisse, un peu froid.
+enfant-m|Une petite fenêtre, oui.
+narrateur|Le ventre de Victorino se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>chaise,voix</t>
         </is>
       </c>
     </row>
@@ -1786,17 +1829,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorino range son cartable. La feuille brune glisse encore dans la poche. La porte rouge s'ouvre. Tu as passé un bon moment ? J'ai montré ma feuille. Elle a un trou. Elle était sur le lait ? Oui, maman. On rentre. La porte rouge se ferme tout doucement. Les feuilles font encore crac. La cuisine sent un peu le pain froid. Victorino pose la feuille sur la table. Près du sel. Oui. Près du sel. On voit bien le trou, maintenant. Un rayon passe dans le trou. Une petite fenêtre. Une toute petite.</t>
+          <t>Plus tard, la porte rouge s'ouvre. Tu as passé un bon moment ? Ma feuille, papa ! Papa n'a pas fini sa phrase. Le sac est près du banc, Victorino. Les deux voix se mélangent. Oh. Victorino refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La feuille est dans ta poche ? Maman n'a pas fini non plus. Victorino reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Ma feuille est brune. Elle a un petit trou. Merci, Victorino. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Victorino veut poser la feuille, tout de suite. Il la saisit trop vite. La feuille glisse entre ses doigts. Oh. Victorino s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la feuille plus lentement. Elle est sèche, maman ! On voit le petit trou. On rentre. Les feuilles font crac sous les chaussures. La porte de la maison s'ouvre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorino range son cartable. La feuille brune glisse encore dans la poche. La porte rouge s'ouvre. Tu as passé un bon moment ? J'ai montré ma feuille. Elle a un trou. Elle était sur le lait ? Oui, maman. On rentre. La porte rouge se ferme tout doucement. Les feuilles font encore crac. La cuisine sent un peu le pain froid. Victorino pose la feuille sur la table. Près du sel. Oui. Près du sel. On voit bien le trou, maintenant. Un rayon passe dans le trou. Une petite fenêtre. Une toute petite.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus tard, la porte rouge s'ouvre. Tu as passé un bon moment ? Ma &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt;, papa ! Papa n'a pas fini sa phrase. Le sac est près du banc, Victorino. Les deux voix se mélangent. Oh. Victorino refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La feuille est dans ta poche ? Maman n'a pas fini non plus. Victorino reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Ma feuille est brune. Elle a un petit trou. Merci, Victorino. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Victorino veut poser la feuille, tout de suite. Il la saisit trop vite. La feuille glisse entre ses doigts. Oh. Victorino s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la feuille plus lentement. Elle est sèche, maman ! On voit le petit trou. On rentre. Les feuilles font crac sous les chaussures. La porte de la maison s'ouvre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dorian range son cartable. Maman l'attend à la porte.&lt;/slow&gt; [pause]</t>
+          <t>Plus tard, la porte rouge s'ouvre. Tu as passé un bon moment ? Ma &lt;emphasis&gt;feuille&lt;/emphasis&gt;, papa ! Papa n'a pas fini sa phrase. Le sac est près du banc, Victorino. Les deux voix se mélangent. Oh. Victorino refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La feuille est dans ta poche ? Maman n'a pas fini non plus. Victorino reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Ma feuille est brune. Elle a un petit trou. Merci, Victorino. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Victorino veut poser la feuille, tout de suite. Il la saisit trop vite. La feuille glisse entre ses doigts. Oh. Victorino s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la feuille plus lentement. Elle est sèche, maman ! On voit le petit trou. On rentre. Les feuilles font crac sous les chaussures. La porte de la maison s'ouvre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1843,18 +1886,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1875,28 +1918,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>feuille</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,10 +1952,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1917,31 +1964,51 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_couper_papa; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Victorino range son cartable.
-narrateur|La feuille brune glisse encore dans la poche.
-narrateur|La porte rouge s'ouvre.
+          <t>narrateur|Plus tard, la porte rouge s'ouvre.
 papa|Tu as passé un bon moment ?
-enfant-m|J'ai montré ma feuille.
-enfant-m|Elle a un trou.
-maman|Elle était sur le lait ?
+enfant-m|Ma feuille, papa !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le sac est près du banc, Victorino.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains à plat.
+papa|Tes pieds sont près de la table ?
+narrateur|Papa pose le sac contre le bois.
+maman|La feuille est dans ta poche ?
+narrateur|Maman n'a pas fini non plus.
+narrateur|Victorino reste jusqu'au silence.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Ma feuille est brune.
+enfant-m|Elle a un petit trou.
+papa|Merci, Victorino.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux un peu d'eau ?
 enfant-m|Oui, maman.
+narrateur|Victorino veut poser la feuille, tout de suite.
+narrateur|Il la saisit trop vite.
+narrateur|La feuille glisse entre ses doigts.
+enfant-m|Oh.
+narrateur|Victorino s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Il pose la feuille plus lentement.
+enfant-m|Elle est sèche, maman !
+maman|On voit le petit trou.
 papa|On rentre.
-narrateur|La porte rouge se ferme tout doucement.
-narrateur|Les feuilles font encore crac.
-narrateur|La cuisine sent un peu le pain froid.
-narrateur|Victorino pose la feuille sur la table.
-enfant-m|Près du sel.
-maman|Oui.
-maman|Près du sel.
-papa|On voit bien le trou, maintenant.
-narrateur|Un rayon passe dans le trou.
-enfant-m|Une petite fenêtre.
-maman|Une toute petite.</t>
+narrateur|Les feuilles font crac sous les chaussures.
+narrateur|La porte de la maison s'ouvre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1973,17 +2040,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La feuille brune dort près du sel. Elle a une petite fenêtre. Bonne soirée, mon grand.</t>
+          <t>Ils restent près de la table. La feuille brune dort près du sel. Comme ce matin, papa ! Tu le vois, le petit trou ? Oui, une petite fenêtre. On est bien, ici. La cuisine sent un peu le toast froid. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Le pain grillé repose dans l'assiette. L'éclat, il est là. On le laisse ? Oui. L'éclat de mie tient sur le toast.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La feuille brune dort près du sel. Elle a une petite fenêtre. Bonne soirée, mon grand.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. La feuille brune dort près du sel. Comme ce matin, papa ! Tu le vois, le petit trou ? Oui, une petite fenêtre. On est bien, ici. La cuisine sent un peu le toast froid. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Le pain grillé repose dans l'assiette. L'éclat, il est là. On le laisse ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de mie&lt;/emphasis&gt; tient sur le toast.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. La feuille brune dort près du sel. Comme ce matin, papa ! Tu le vois, le petit trou ? Oui, une petite fenêtre. On est bien, ici. La cuisine sent un peu le toast froid. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Le pain grillé repose dans l'assiette. L'éclat, il est là. On le laisse ? Oui. L'&lt;emphasis&gt;éclat de mie&lt;/emphasis&gt; tient sur le toast.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2030,7 +2097,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2038,10 +2105,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2050,12 +2117,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2064,17 +2131,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de mie</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2083,11 +2154,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2096,26 +2167,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_toast; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La feuille brune dort près du sel.
-maman|Elle a une petite fenêtre.
-papa|Bonne soirée, mon grand.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|La feuille brune dort près du sel.
+enfant-m|Comme ce matin, papa !
+papa|Tu le vois, le petit trou ?
+enfant-m|Oui, une petite fenêtre.
+maman|On est bien, ici.
+narrateur|La cuisine sent un peu le toast froid.
+narrateur|Victorino glisse le pied, sans se presser.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est tiède.
+narrateur|Le pain grillé repose dans l'assiette.
+enfant-m|L'éclat, il est là.
+papa|On le laisse ?
+enfant-m|Oui.
+narrateur|L'éclat de mie tient sur le toast.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>toast,feuille</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2221,6 +2314,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>